<commit_message>
Add configurable special value profiling and numeric percentiles
</commit_message>
<xml_diff>
--- a/DQ_ENGINE/config/DQ_RDS_config.xlsx
+++ b/DQ_ENGINE/config/DQ_RDS_config.xlsx
@@ -5,6 +5,7 @@
     <sheet name="Project" sheetId="1" r:id="rId1"/>
     <sheet name="Fields" sheetId="2" r:id="rId2"/>
     <sheet name="Settings" sheetId="3" r:id="rId3"/>
+    <sheet name="SpecialValues" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -10241,4 +10242,579 @@
   </sheetData>
   <autoFilter ref="A1:D2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:C33"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>FIELD_TYPE</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>SPECIAL_VALUE</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>ACTIVE_IND</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>NUMERIC</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>-99999</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NUMERIC</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>-999999</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>NUMERIC</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>-999998</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>NUMERIC</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>-99998</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>NUMERIC</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>-99997</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>NUMERIC</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>-9999</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>NUMERIC</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>-9998</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>NUMERIC</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>-999997</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>NUMERIC</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>-999993</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>NUMERIC</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>-999</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>NUMERIC</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>-999995</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>NUMERIC</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>999999</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>NUMERIC</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>999998</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>NUMERIC</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>999990</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>NUMERIC</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>99999</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>NUMERIC</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>99998</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>NUMERIC</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>999.99</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>NUMERIC</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>999.88</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>NUMERIC</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>999</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>NUMERIC</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>9999</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>NUMERIC</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>9998</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>CATEGORICAL</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>CATEGORICAL</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>CATEGORICAL</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>CATEGORICAL</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>CATEGORICAL</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>CATEGORICAL</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>CATEGORICAL</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>CATEGORICAL</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>#N/A</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>CATEGORICAL</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>CATEGORICAL</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>CATEGORICAL</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>NOT APPLICABLE</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C33"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Configure profiling reporting levels independently of modules
</commit_message>
<xml_diff>
--- a/DQ_ENGINE/config/DQ_RDS_config.xlsx
+++ b/DQ_ENGINE/config/DQ_RDS_config.xlsx
@@ -10195,12 +10195,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:G2"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
     <col min="4" max="4" width="24" customWidth="1"/>
+    <col min="5" max="7" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10224,6 +10225,21 @@
           <t>OUTLIER_SD_MULTIPLIER</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t>PROFILE_OVERALL</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
+          <t>PROFILE_MONTHLY</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
+          <t>PROFILE_YEARLY</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -10238,9 +10254,29 @@
       <c r="D2">
         <v>3</v>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D2"/>
+  <autoFilter ref="A1:G2"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Choose Y or N" error="Select Y or N." sqref="E2:G2">
+      <formula1>"Y,N"</formula1>
+    </dataValidation>
+  </dataValidations>
 </worksheet>
 </file>
 

</xml_diff>